<commit_message>
Final Fix: Global scope for MediaPipe and Ellipse calibration
</commit_message>
<xml_diff>
--- a/Mẫu số đo & Đánh giá Model CV.xlsx
+++ b/Mẫu số đo & Đánh giá Model CV.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lap_Trinh_2022-2026-20230924T092707Z-001\Bodyfat_predict\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B49FE6C-52D8-4881-9DD6-2BD0B8C50CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B4DAFFE-D88A-46F8-AF4C-EF67B48455E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="13667" xr2:uid="{F2E29C3A-FB58-4893-8DD4-400619C0E675}"/>
+    <workbookView xWindow="5485" yWindow="2985" windowWidth="14937" windowHeight="7370" xr2:uid="{F2E29C3A-FB58-4893-8DD4-400619C0E675}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1135,25 +1135,25 @@
         <v>86</v>
       </c>
       <c r="G2" s="1">
-        <v>82.06</v>
+        <v>88.62</v>
       </c>
       <c r="H2">
         <v>74</v>
       </c>
       <c r="I2" s="1">
-        <v>59.96</v>
+        <v>79.650000000000006</v>
       </c>
       <c r="J2">
         <v>90</v>
       </c>
       <c r="K2" s="1">
-        <v>83.13</v>
+        <v>91.32</v>
       </c>
       <c r="L2">
         <v>50</v>
       </c>
       <c r="M2" s="1">
-        <v>39.79</v>
+        <v>42.97</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">

</xml_diff>